<commit_message>
Update arbeidsplan Excel from SharePoint
</commit_message>
<xml_diff>
--- a/input/Arbeidsplan simulatoroperatører.xlsx
+++ b/input/Arbeidsplan simulatoroperatører.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://avinor.sharepoint.com/sites/GRP_Simulatordrift_avd.Vaernes/Delte dokumenter/General/Arbeidsplaner/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3692" documentId="8_{95B923E9-95EE-4F78-B225-2EDB4F75667E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6096BA85-98AF-4A65-98DD-CC96308A0228}"/>
+  <xr:revisionPtr revIDLastSave="3751" documentId="8_{95B923E9-95EE-4F78-B225-2EDB4F75667E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85046D33-AC8E-4594-A833-5284DF811392}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="lgNItpb0Ti65q+mfEUdHXTOz24BuywDWtkFml2UWap2uCRRSwJcP050KCJ16GV7eXwgKeIkDdd7RYQr9U+X8Rw==" workbookSaltValue="526Uxco+d+5gCLKuUY2fsw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Uke 1-6" sheetId="7" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3311" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3297" uniqueCount="237">
   <si>
     <t>Uke 01</t>
   </si>
@@ -757,6 +757,9 @@
   <si>
     <t>9 SF ADC</t>
   </si>
+  <si>
+    <t>Pilot BO</t>
+  </si>
 </sst>
 </file>
 
@@ -1035,7 +1038,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1285,12 +1288,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1307,6 +1304,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -11039,7 +11039,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AI60"/>
+  <dimension ref="A1:X60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" style="4" bestFit="1" customWidth="1"/>
@@ -11489,22 +11489,22 @@
       </c>
       <c r="O9" s="77"/>
       <c r="P9" s="78"/>
-      <c r="Q9" s="87" t="s">
+      <c r="Q9" s="85" t="s">
         <v>229</v>
       </c>
-      <c r="R9" s="88"/>
-      <c r="S9" s="87" t="s">
+      <c r="R9" s="86"/>
+      <c r="S9" s="85" t="s">
         <v>229</v>
       </c>
-      <c r="T9" s="88"/>
-      <c r="U9" s="87" t="s">
+      <c r="T9" s="86"/>
+      <c r="U9" s="85" t="s">
         <v>229</v>
       </c>
-      <c r="V9" s="88"/>
-      <c r="W9" s="87" t="s">
+      <c r="V9" s="86"/>
+      <c r="W9" s="85" t="s">
         <v>229</v>
       </c>
-      <c r="X9" s="88"/>
+      <c r="X9" s="86"/>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
@@ -11673,22 +11673,22 @@
       </c>
       <c r="O13" s="77"/>
       <c r="P13" s="78"/>
-      <c r="Q13" s="87" t="s">
+      <c r="Q13" s="85" t="s">
         <v>171</v>
       </c>
-      <c r="R13" s="88"/>
-      <c r="S13" s="87" t="s">
+      <c r="R13" s="86"/>
+      <c r="S13" s="85" t="s">
         <v>171</v>
       </c>
-      <c r="T13" s="88"/>
-      <c r="U13" s="87" t="s">
+      <c r="T13" s="86"/>
+      <c r="U13" s="85" t="s">
         <v>171</v>
       </c>
-      <c r="V13" s="88"/>
-      <c r="W13" s="87" t="s">
+      <c r="V13" s="86"/>
+      <c r="W13" s="85" t="s">
         <v>171</v>
       </c>
-      <c r="X13" s="88"/>
+      <c r="X13" s="86"/>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
@@ -12102,26 +12102,26 @@
       <c r="N24" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="O24" s="87" t="s">
+      <c r="O24" s="85" t="s">
         <v>171</v>
       </c>
-      <c r="P24" s="88"/>
-      <c r="Q24" s="87" t="s">
+      <c r="P24" s="86"/>
+      <c r="Q24" s="85" t="s">
         <v>171</v>
       </c>
-      <c r="R24" s="88"/>
-      <c r="S24" s="87" t="s">
+      <c r="R24" s="86"/>
+      <c r="S24" s="85" t="s">
         <v>171</v>
       </c>
-      <c r="T24" s="88"/>
-      <c r="U24" s="87" t="s">
+      <c r="T24" s="86"/>
+      <c r="U24" s="85" t="s">
         <v>171</v>
       </c>
-      <c r="V24" s="88"/>
-      <c r="W24" s="87" t="s">
+      <c r="V24" s="86"/>
+      <c r="W24" s="85" t="s">
         <v>171</v>
       </c>
-      <c r="X24" s="88"/>
+      <c r="X24" s="86"/>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
@@ -12240,26 +12240,26 @@
       <c r="N27" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="O27" s="87" t="s">
+      <c r="O27" s="85" t="s">
         <v>229</v>
       </c>
-      <c r="P27" s="88"/>
-      <c r="Q27" s="87" t="s">
+      <c r="P27" s="86"/>
+      <c r="Q27" s="85" t="s">
         <v>229</v>
       </c>
-      <c r="R27" s="88"/>
-      <c r="S27" s="87" t="s">
+      <c r="R27" s="86"/>
+      <c r="S27" s="85" t="s">
         <v>229</v>
       </c>
-      <c r="T27" s="88"/>
-      <c r="U27" s="87" t="s">
+      <c r="T27" s="86"/>
+      <c r="U27" s="85" t="s">
         <v>229</v>
       </c>
-      <c r="V27" s="88"/>
-      <c r="W27" s="87" t="s">
+      <c r="V27" s="86"/>
+      <c r="W27" s="85" t="s">
         <v>229</v>
       </c>
-      <c r="X27" s="88"/>
+      <c r="X27" s="86"/>
     </row>
     <row r="28" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A28" s="6" t="s">
@@ -12495,7 +12495,7 @@
       </c>
       <c r="X32" s="40"/>
     </row>
-    <row r="33" spans="1:35" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>48</v>
       </c>
@@ -12543,7 +12543,7 @@
       </c>
       <c r="X33" s="18"/>
     </row>
-    <row r="34" spans="1:35" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A34" s="12" t="s">
         <v>49</v>
       </c>
@@ -12591,7 +12591,7 @@
       </c>
       <c r="X34" s="40"/>
     </row>
-    <row r="35" spans="1:35" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>50</v>
       </c>
@@ -12633,7 +12633,7 @@
       </c>
       <c r="X35" s="18"/>
     </row>
-    <row r="36" spans="1:35" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:24" x14ac:dyDescent="0.2">
       <c r="L36" s="7"/>
       <c r="M36" s="7"/>
       <c r="N36" s="4"/>
@@ -12641,7 +12641,7 @@
       <c r="Q36" s="4"/>
       <c r="R36" s="4"/>
     </row>
-    <row r="37" spans="1:35" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:24" x14ac:dyDescent="0.2">
       <c r="L37" s="7"/>
       <c r="M37" s="7"/>
       <c r="N37" s="4"/>
@@ -12649,7 +12649,7 @@
       <c r="Q37" s="4"/>
       <c r="R37" s="4"/>
     </row>
-    <row r="38" spans="1:35" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:24" x14ac:dyDescent="0.2">
       <c r="L38" s="7"/>
       <c r="M38" s="7"/>
       <c r="N38" s="4"/>
@@ -12657,7 +12657,7 @@
       <c r="Q38" s="4"/>
       <c r="R38" s="4"/>
     </row>
-    <row r="39" spans="1:35" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>182</v>
       </c>
@@ -12727,7 +12727,7 @@
         <v>46185</v>
       </c>
     </row>
-    <row r="40" spans="1:35" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>7</v>
       </c>
@@ -12777,7 +12777,7 @@
       </c>
       <c r="X40" s="46"/>
     </row>
-    <row r="41" spans="1:35" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>10</v>
       </c>
@@ -12810,36 +12810,24 @@
         <v>8</v>
       </c>
       <c r="P41" s="38"/>
-      <c r="Q41" s="43"/>
-      <c r="R41" s="44"/>
-      <c r="S41" s="43"/>
-      <c r="T41" s="44"/>
-      <c r="U41" s="17"/>
+      <c r="Q41" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="R41" s="18"/>
+      <c r="S41" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="T41" s="18"/>
+      <c r="U41" s="17" t="s">
+        <v>169</v>
+      </c>
       <c r="V41" s="18"/>
-      <c r="W41" s="17"/>
+      <c r="W41" s="17" t="s">
+        <v>169</v>
+      </c>
       <c r="X41" s="18"/>
-      <c r="Z41" s="37" t="s">
-        <v>8</v>
-      </c>
-      <c r="AA41" s="38"/>
-      <c r="AB41" s="43" t="s">
-        <v>181</v>
-      </c>
-      <c r="AC41" s="44"/>
-      <c r="AD41" s="43" t="s">
-        <v>181</v>
-      </c>
-      <c r="AE41" s="44"/>
-      <c r="AF41" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="AG41" s="18"/>
-      <c r="AH41" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="AI41" s="18"/>
-    </row>
-    <row r="42" spans="1:35" x14ac:dyDescent="0.2">
+    </row>
+    <row r="42" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>15</v>
       </c>
@@ -12868,38 +12856,28 @@
       <c r="N42" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="O42" s="69"/>
+      <c r="O42" s="69" t="s">
+        <v>149</v>
+      </c>
       <c r="P42" s="70"/>
-      <c r="Q42" s="69"/>
+      <c r="Q42" s="69" t="s">
+        <v>149</v>
+      </c>
       <c r="R42" s="70"/>
-      <c r="S42" s="69"/>
+      <c r="S42" s="69" t="s">
+        <v>149</v>
+      </c>
       <c r="T42" s="70"/>
-      <c r="U42" s="17"/>
-      <c r="V42" s="18"/>
-      <c r="W42" s="17"/>
-      <c r="X42" s="18"/>
-      <c r="Z42" s="69" t="s">
-        <v>156</v>
-      </c>
-      <c r="AA42" s="70"/>
-      <c r="AB42" s="69" t="s">
-        <v>156</v>
-      </c>
-      <c r="AC42" s="70"/>
-      <c r="AD42" s="69" t="s">
-        <v>156</v>
-      </c>
-      <c r="AE42" s="70"/>
-      <c r="AF42" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="AG42" s="18"/>
-      <c r="AH42" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="AI42" s="18"/>
-    </row>
-    <row r="43" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="U42" s="33" t="s">
+        <v>151</v>
+      </c>
+      <c r="V42" s="34"/>
+      <c r="W42" s="33" t="s">
+        <v>151</v>
+      </c>
+      <c r="X42" s="34"/>
+    </row>
+    <row r="43" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>21</v>
       </c>
@@ -12926,38 +12904,28 @@
       <c r="N43" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="O43" s="17"/>
-      <c r="P43" s="18"/>
-      <c r="Q43" s="17"/>
-      <c r="R43" s="18"/>
-      <c r="S43" s="17"/>
-      <c r="T43" s="18"/>
-      <c r="U43" s="17"/>
-      <c r="V43" s="18"/>
-      <c r="W43" s="17"/>
-      <c r="X43" s="18"/>
-      <c r="Z43" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="AA43" s="18"/>
-      <c r="AB43" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="AC43" s="18"/>
-      <c r="AD43" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="AE43" s="18"/>
-      <c r="AF43" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="AG43" s="18"/>
-      <c r="AH43" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="AI43" s="18"/>
-    </row>
-    <row r="44" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="O43" s="39" t="s">
+        <v>165</v>
+      </c>
+      <c r="P43" s="40"/>
+      <c r="Q43" s="39" t="s">
+        <v>165</v>
+      </c>
+      <c r="R43" s="40"/>
+      <c r="S43" s="39" t="s">
+        <v>165</v>
+      </c>
+      <c r="T43" s="40"/>
+      <c r="U43" s="39" t="s">
+        <v>165</v>
+      </c>
+      <c r="V43" s="40"/>
+      <c r="W43" s="39" t="s">
+        <v>165</v>
+      </c>
+      <c r="X43" s="40"/>
+    </row>
+    <row r="44" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>24</v>
       </c>
@@ -12965,14 +12933,14 @@
         <v>91</v>
       </c>
       <c r="C44" s="44"/>
-      <c r="D44" s="89" t="s">
+      <c r="D44" s="87" t="s">
         <v>185</v>
       </c>
-      <c r="E44" s="90"/>
-      <c r="F44" s="89" t="s">
+      <c r="E44" s="88"/>
+      <c r="F44" s="87" t="s">
         <v>184</v>
       </c>
-      <c r="G44" s="90"/>
+      <c r="G44" s="88"/>
       <c r="H44" s="43" t="s">
         <v>91</v>
       </c>
@@ -13004,86 +12972,56 @@
         <v>91</v>
       </c>
       <c r="X44" s="44"/>
-      <c r="Z44" s="43" t="s">
-        <v>91</v>
-      </c>
-      <c r="AA44" s="44"/>
-      <c r="AB44" s="43" t="s">
-        <v>91</v>
-      </c>
-      <c r="AC44" s="44"/>
-      <c r="AD44" s="43" t="s">
-        <v>91</v>
-      </c>
-      <c r="AE44" s="44"/>
-      <c r="AF44" s="43" t="s">
-        <v>91</v>
-      </c>
-      <c r="AG44" s="44"/>
-      <c r="AH44" s="43" t="s">
-        <v>91</v>
-      </c>
-      <c r="AI44" s="44"/>
-    </row>
-    <row r="45" spans="1:35" x14ac:dyDescent="0.2">
+    </row>
+    <row r="45" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A45" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B45" s="87" t="s">
+      <c r="B45" s="85" t="s">
         <v>229</v>
       </c>
-      <c r="C45" s="88"/>
-      <c r="D45" s="87" t="s">
+      <c r="C45" s="86"/>
+      <c r="D45" s="85" t="s">
         <v>230</v>
       </c>
-      <c r="E45" s="88"/>
-      <c r="F45" s="87" t="s">
+      <c r="E45" s="86"/>
+      <c r="F45" s="85" t="s">
         <v>229</v>
       </c>
-      <c r="G45" s="88"/>
-      <c r="H45" s="87" t="s">
+      <c r="G45" s="86"/>
+      <c r="H45" s="85" t="s">
         <v>229</v>
       </c>
-      <c r="I45" s="88"/>
-      <c r="J45" s="87" t="s">
+      <c r="I45" s="86"/>
+      <c r="J45" s="85" t="s">
         <v>229</v>
       </c>
-      <c r="K45" s="88"/>
+      <c r="K45" s="86"/>
       <c r="N45" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="O45" s="17"/>
-      <c r="P45" s="18"/>
-      <c r="Q45" s="17"/>
-      <c r="R45" s="18"/>
-      <c r="S45" s="17"/>
-      <c r="T45" s="18"/>
-      <c r="U45" s="39"/>
-      <c r="V45" s="40"/>
-      <c r="W45" s="39"/>
-      <c r="X45" s="40"/>
-      <c r="Z45" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="AA45" s="18"/>
-      <c r="AB45" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="AC45" s="18"/>
-      <c r="AD45" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="AE45" s="18"/>
-      <c r="AF45" s="39" t="s">
-        <v>163</v>
-      </c>
-      <c r="AG45" s="40"/>
-      <c r="AH45" s="39" t="s">
-        <v>163</v>
-      </c>
-      <c r="AI45" s="40"/>
-    </row>
-    <row r="46" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="O45" s="69" t="s">
+        <v>156</v>
+      </c>
+      <c r="P45" s="70"/>
+      <c r="Q45" s="69" t="s">
+        <v>156</v>
+      </c>
+      <c r="R45" s="70"/>
+      <c r="S45" s="69" t="s">
+        <v>156</v>
+      </c>
+      <c r="T45" s="70"/>
+      <c r="U45" s="33" t="s">
+        <v>150</v>
+      </c>
+      <c r="V45" s="34"/>
+      <c r="W45" s="33" t="s">
+        <v>150</v>
+      </c>
+      <c r="X45" s="34"/>
+    </row>
+    <row r="46" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A46" s="6" t="s">
         <v>28</v>
       </c>
@@ -13091,14 +13029,14 @@
         <v>165</v>
       </c>
       <c r="C46" s="40"/>
-      <c r="D46" s="89" t="s">
+      <c r="D46" s="87" t="s">
         <v>233</v>
       </c>
-      <c r="E46" s="90"/>
-      <c r="F46" s="89" t="s">
+      <c r="E46" s="88"/>
+      <c r="F46" s="87" t="s">
         <v>234</v>
       </c>
-      <c r="G46" s="90"/>
+      <c r="G46" s="88"/>
       <c r="H46" s="29" t="s">
         <v>9</v>
       </c>
@@ -13110,61 +13048,51 @@
       <c r="N46" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="O46" s="39"/>
-      <c r="P46" s="40"/>
-      <c r="Q46" s="39"/>
-      <c r="R46" s="40"/>
-      <c r="S46" s="39"/>
-      <c r="T46" s="40"/>
-      <c r="U46" s="39"/>
-      <c r="V46" s="40"/>
-      <c r="W46" s="39"/>
-      <c r="X46" s="40"/>
-      <c r="Z46" s="39" t="s">
-        <v>163</v>
-      </c>
-      <c r="AA46" s="40"/>
-      <c r="AB46" s="39" t="s">
-        <v>163</v>
-      </c>
-      <c r="AC46" s="40"/>
-      <c r="AD46" s="39" t="s">
-        <v>163</v>
-      </c>
-      <c r="AE46" s="40"/>
-      <c r="AF46" s="39" t="s">
-        <v>163</v>
-      </c>
-      <c r="AG46" s="40"/>
-      <c r="AH46" s="39" t="s">
-        <v>163</v>
-      </c>
-      <c r="AI46" s="40"/>
-    </row>
-    <row r="47" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="O46" s="23" t="s">
+        <v>223</v>
+      </c>
+      <c r="P46" s="24"/>
+      <c r="Q46" s="23" t="s">
+        <v>224</v>
+      </c>
+      <c r="R46" s="24"/>
+      <c r="S46" s="23" t="s">
+        <v>224</v>
+      </c>
+      <c r="T46" s="24"/>
+      <c r="U46" s="23" t="s">
+        <v>224</v>
+      </c>
+      <c r="V46" s="24"/>
+      <c r="W46" s="23" t="s">
+        <v>224</v>
+      </c>
+      <c r="X46" s="24"/>
+    </row>
+    <row r="47" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A47" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B47" s="87" t="s">
+      <c r="B47" s="85" t="s">
         <v>171</v>
       </c>
-      <c r="C47" s="88"/>
-      <c r="D47" s="87" t="s">
+      <c r="C47" s="86"/>
+      <c r="D47" s="85" t="s">
         <v>186</v>
       </c>
-      <c r="E47" s="88"/>
-      <c r="F47" s="87" t="s">
+      <c r="E47" s="86"/>
+      <c r="F47" s="85" t="s">
         <v>171</v>
       </c>
-      <c r="G47" s="88"/>
-      <c r="H47" s="87" t="s">
+      <c r="G47" s="86"/>
+      <c r="H47" s="85" t="s">
         <v>171</v>
       </c>
-      <c r="I47" s="88"/>
-      <c r="J47" s="87" t="s">
+      <c r="I47" s="86"/>
+      <c r="J47" s="85" t="s">
         <v>171</v>
       </c>
-      <c r="K47" s="88"/>
+      <c r="K47" s="86"/>
       <c r="N47" s="6" t="s">
         <v>32</v>
       </c>
@@ -13188,28 +13116,8 @@
         <v>8</v>
       </c>
       <c r="X47" s="38"/>
-      <c r="Z47" s="37" t="s">
-        <v>8</v>
-      </c>
-      <c r="AA47" s="38"/>
-      <c r="AB47" s="37" t="s">
-        <v>8</v>
-      </c>
-      <c r="AC47" s="38"/>
-      <c r="AD47" s="37" t="s">
-        <v>8</v>
-      </c>
-      <c r="AE47" s="38"/>
-      <c r="AF47" s="37" t="s">
-        <v>8</v>
-      </c>
-      <c r="AG47" s="38"/>
-      <c r="AH47" s="37" t="s">
-        <v>8</v>
-      </c>
-      <c r="AI47" s="38"/>
-    </row>
-    <row r="48" spans="1:35" x14ac:dyDescent="0.2">
+    </row>
+    <row r="48" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A48" s="6" t="s">
         <v>35</v>
       </c>
@@ -13236,38 +13144,28 @@
       <c r="N48" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="O48" s="39"/>
+      <c r="O48" s="39" t="s">
+        <v>163</v>
+      </c>
       <c r="P48" s="40"/>
-      <c r="Q48" s="39"/>
+      <c r="Q48" s="39" t="s">
+        <v>163</v>
+      </c>
       <c r="R48" s="40"/>
-      <c r="S48" s="39"/>
+      <c r="S48" s="39" t="s">
+        <v>163</v>
+      </c>
       <c r="T48" s="40"/>
-      <c r="U48" s="23"/>
-      <c r="V48" s="24"/>
-      <c r="W48" s="23"/>
-      <c r="X48" s="24"/>
-      <c r="Z48" s="39" t="s">
+      <c r="U48" s="39" t="s">
         <v>163</v>
       </c>
-      <c r="AA48" s="40"/>
-      <c r="AB48" s="39" t="s">
+      <c r="V48" s="40"/>
+      <c r="W48" s="39" t="s">
         <v>163</v>
       </c>
-      <c r="AC48" s="40"/>
-      <c r="AD48" s="39" t="s">
-        <v>163</v>
-      </c>
-      <c r="AE48" s="40"/>
-      <c r="AF48" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="AG48" s="24"/>
-      <c r="AH48" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="AI48" s="24"/>
-    </row>
-    <row r="49" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="X48" s="40"/>
+    </row>
+    <row r="49" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>37</v>
       </c>
@@ -13294,38 +13192,28 @@
       <c r="N49" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="O49" s="39"/>
-      <c r="P49" s="40"/>
-      <c r="Q49" s="39"/>
-      <c r="R49" s="40"/>
-      <c r="S49" s="39"/>
-      <c r="T49" s="40"/>
-      <c r="U49" s="33"/>
+      <c r="O49" s="43" t="s">
+        <v>235</v>
+      </c>
+      <c r="P49" s="44"/>
+      <c r="Q49" s="43" t="s">
+        <v>235</v>
+      </c>
+      <c r="R49" s="44"/>
+      <c r="S49" s="43" t="s">
+        <v>235</v>
+      </c>
+      <c r="T49" s="44"/>
+      <c r="U49" s="33" t="s">
+        <v>151</v>
+      </c>
       <c r="V49" s="34"/>
-      <c r="W49" s="33"/>
+      <c r="W49" s="33" t="s">
+        <v>151</v>
+      </c>
       <c r="X49" s="34"/>
-      <c r="Z49" s="39" t="s">
-        <v>163</v>
-      </c>
-      <c r="AA49" s="40"/>
-      <c r="AB49" s="39" t="s">
-        <v>163</v>
-      </c>
-      <c r="AC49" s="40"/>
-      <c r="AD49" s="39" t="s">
-        <v>163</v>
-      </c>
-      <c r="AE49" s="40"/>
-      <c r="AF49" s="33" t="s">
-        <v>151</v>
-      </c>
-      <c r="AG49" s="34"/>
-      <c r="AH49" s="33" t="s">
-        <v>151</v>
-      </c>
-      <c r="AI49" s="34"/>
-    </row>
-    <row r="50" spans="1:35" x14ac:dyDescent="0.2">
+    </row>
+    <row r="50" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>40</v>
       </c>
@@ -13354,38 +13242,28 @@
       <c r="N50" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="O50" s="23"/>
-      <c r="P50" s="24"/>
-      <c r="Q50" s="23"/>
-      <c r="R50" s="24"/>
-      <c r="S50" s="23"/>
-      <c r="T50" s="24"/>
-      <c r="U50" s="33"/>
-      <c r="V50" s="34"/>
-      <c r="W50" s="33"/>
-      <c r="X50" s="34"/>
-      <c r="Z50" s="23" t="s">
-        <v>136</v>
-      </c>
-      <c r="AA50" s="24"/>
-      <c r="AB50" s="23" t="s">
-        <v>136</v>
-      </c>
-      <c r="AC50" s="24"/>
-      <c r="AD50" s="23" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE50" s="24"/>
-      <c r="AF50" s="33" t="s">
-        <v>151</v>
-      </c>
-      <c r="AG50" s="34"/>
-      <c r="AH50" s="33" t="s">
-        <v>151</v>
-      </c>
-      <c r="AI50" s="34"/>
-    </row>
-    <row r="51" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="O50" s="17" t="s">
+        <v>227</v>
+      </c>
+      <c r="P50" s="18"/>
+      <c r="Q50" s="17" t="s">
+        <v>227</v>
+      </c>
+      <c r="R50" s="18"/>
+      <c r="S50" s="17" t="s">
+        <v>227</v>
+      </c>
+      <c r="T50" s="18"/>
+      <c r="U50" s="17" t="s">
+        <v>227</v>
+      </c>
+      <c r="V50" s="18"/>
+      <c r="W50" s="17" t="s">
+        <v>227</v>
+      </c>
+      <c r="X50" s="18"/>
+    </row>
+    <row r="51" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A51" s="12" t="s">
         <v>45</v>
       </c>
@@ -13414,38 +13292,28 @@
       <c r="N51" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="O51" s="23"/>
+      <c r="O51" s="23" t="s">
+        <v>136</v>
+      </c>
       <c r="P51" s="24"/>
-      <c r="Q51" s="23"/>
+      <c r="Q51" s="23" t="s">
+        <v>136</v>
+      </c>
       <c r="R51" s="24"/>
-      <c r="S51" s="23"/>
+      <c r="S51" s="23" t="s">
+        <v>136</v>
+      </c>
       <c r="T51" s="24"/>
-      <c r="U51" s="33"/>
-      <c r="V51" s="34"/>
-      <c r="W51" s="33"/>
-      <c r="X51" s="34"/>
-      <c r="Z51" s="23" t="s">
-        <v>140</v>
-      </c>
-      <c r="AA51" s="24"/>
-      <c r="AB51" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="AC51" s="24"/>
-      <c r="AD51" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="AE51" s="24"/>
-      <c r="AF51" s="33" t="s">
-        <v>151</v>
-      </c>
-      <c r="AG51" s="34"/>
-      <c r="AH51" s="33" t="s">
-        <v>151</v>
-      </c>
-      <c r="AI51" s="34"/>
-    </row>
-    <row r="52" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="U51" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="V51" s="18"/>
+      <c r="W51" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="X51" s="18"/>
+    </row>
+    <row r="52" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>48</v>
       </c>
@@ -13474,34 +13342,28 @@
       <c r="N52" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="O52" s="43"/>
-      <c r="P52" s="44"/>
-      <c r="Q52" s="43"/>
-      <c r="R52" s="44"/>
-      <c r="S52" s="43"/>
-      <c r="T52" s="44"/>
-      <c r="U52" s="29"/>
-      <c r="V52" s="30"/>
-      <c r="W52" s="29"/>
-      <c r="X52" s="30"/>
-      <c r="Z52" s="43" t="s">
-        <v>181</v>
-      </c>
-      <c r="AA52" s="44"/>
-      <c r="AB52" s="43" t="s">
-        <v>181</v>
-      </c>
-      <c r="AC52" s="44"/>
-      <c r="AD52" s="43" t="s">
-        <v>181</v>
-      </c>
-      <c r="AE52" s="44"/>
-      <c r="AF52" s="29"/>
-      <c r="AG52" s="30"/>
-      <c r="AH52" s="29"/>
-      <c r="AI52" s="30"/>
-    </row>
-    <row r="53" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="O52" s="39" t="s">
+        <v>163</v>
+      </c>
+      <c r="P52" s="40"/>
+      <c r="Q52" s="39" t="s">
+        <v>163</v>
+      </c>
+      <c r="R52" s="40"/>
+      <c r="S52" s="39" t="s">
+        <v>163</v>
+      </c>
+      <c r="T52" s="40"/>
+      <c r="U52" s="39" t="s">
+        <v>163</v>
+      </c>
+      <c r="V52" s="40"/>
+      <c r="W52" s="39" t="s">
+        <v>163</v>
+      </c>
+      <c r="X52" s="40"/>
+    </row>
+    <row r="53" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A53" s="12" t="s">
         <v>49</v>
       </c>
@@ -13528,8 +13390,10 @@
       <c r="N53" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="O53" s="43"/>
-      <c r="P53" s="44"/>
+      <c r="O53" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="P53" s="18"/>
       <c r="Q53" s="37" t="s">
         <v>8</v>
       </c>
@@ -13546,28 +13410,8 @@
         <v>8</v>
       </c>
       <c r="X53" s="38"/>
-      <c r="Z53" s="43" t="s">
-        <v>181</v>
-      </c>
-      <c r="AA53" s="44"/>
-      <c r="AB53" s="37" t="s">
-        <v>8</v>
-      </c>
-      <c r="AC53" s="38"/>
-      <c r="AD53" s="37" t="s">
-        <v>8</v>
-      </c>
-      <c r="AE53" s="38"/>
-      <c r="AF53" s="37" t="s">
-        <v>8</v>
-      </c>
-      <c r="AG53" s="38"/>
-      <c r="AH53" s="37" t="s">
-        <v>8</v>
-      </c>
-      <c r="AI53" s="38"/>
-    </row>
-    <row r="54" spans="1:35" x14ac:dyDescent="0.2">
+    </row>
+    <row r="54" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>50</v>
       </c>
@@ -13592,34 +13436,24 @@
       <c r="N54" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="O54" s="69"/>
-      <c r="P54" s="70"/>
-      <c r="Q54" s="69"/>
-      <c r="R54" s="70"/>
-      <c r="S54" s="69"/>
-      <c r="T54" s="70"/>
+      <c r="O54" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="P54" s="18"/>
+      <c r="Q54" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="R54" s="18"/>
+      <c r="S54" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="T54" s="18"/>
       <c r="U54" s="29"/>
       <c r="V54" s="30"/>
       <c r="W54" s="29"/>
       <c r="X54" s="30"/>
-      <c r="Z54" s="69" t="s">
-        <v>156</v>
-      </c>
-      <c r="AA54" s="70"/>
-      <c r="AB54" s="69" t="s">
-        <v>156</v>
-      </c>
-      <c r="AC54" s="70"/>
-      <c r="AD54" s="69" t="s">
-        <v>156</v>
-      </c>
-      <c r="AE54" s="70"/>
-      <c r="AF54" s="29"/>
-      <c r="AG54" s="30"/>
-      <c r="AH54" s="29"/>
-      <c r="AI54" s="30"/>
-    </row>
-    <row r="55" spans="1:35" x14ac:dyDescent="0.2">
+    </row>
+    <row r="55" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A55" s="8"/>
       <c r="B55" s="5"/>
       <c r="C55" s="5"/>
@@ -13631,38 +13465,27 @@
       <c r="K55" s="5"/>
       <c r="L55" s="7"/>
       <c r="M55" s="7"/>
-      <c r="O55" s="17"/>
-      <c r="P55" s="18"/>
-      <c r="Q55" s="85"/>
-      <c r="R55" s="86"/>
-      <c r="S55" s="17"/>
-      <c r="T55" s="18"/>
-      <c r="U55" s="39"/>
-      <c r="V55" s="40"/>
-      <c r="W55" s="39"/>
-      <c r="X55" s="40"/>
-      <c r="Z55" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="AA55" s="18"/>
-      <c r="AB55" s="85" t="s">
-        <v>169</v>
-      </c>
-      <c r="AC55" s="86"/>
-      <c r="AD55" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="AE55" s="18"/>
-      <c r="AF55" s="39" t="s">
-        <v>163</v>
-      </c>
-      <c r="AG55" s="40"/>
-      <c r="AH55" s="39" t="s">
-        <v>163</v>
-      </c>
-      <c r="AI55" s="40"/>
-    </row>
-    <row r="56" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="N55" s="12" t="s">
+        <v>236</v>
+      </c>
+      <c r="O55" s="91" t="s">
+        <v>181</v>
+      </c>
+      <c r="P55" s="91"/>
+      <c r="Q55" s="91" t="s">
+        <v>181</v>
+      </c>
+      <c r="R55" s="91"/>
+      <c r="S55" s="91" t="s">
+        <v>181</v>
+      </c>
+      <c r="T55" s="91"/>
+      <c r="U55" s="29"/>
+      <c r="V55" s="30"/>
+      <c r="W55" s="29"/>
+      <c r="X55" s="30"/>
+    </row>
+    <row r="56" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A56" s="8"/>
       <c r="B56" s="5"/>
       <c r="C56" s="5"/>
@@ -13675,7 +13498,7 @@
       <c r="L56" s="7"/>
       <c r="M56" s="7"/>
     </row>
-    <row r="57" spans="1:35" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A57" s="5">
         <v>1</v>
       </c>
@@ -13700,7 +13523,7 @@
       <c r="W57" s="4"/>
       <c r="X57" s="4"/>
     </row>
-    <row r="58" spans="1:35" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A58" s="5">
         <v>2</v>
       </c>
@@ -13714,7 +13537,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="59" spans="1:35" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A59" s="8">
         <v>3</v>
       </c>
@@ -13728,7 +13551,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="60" spans="1:35" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A60" s="5">
         <v>4</v>
       </c>
@@ -13737,82 +13560,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="535">
-    <mergeCell ref="Z55:AA55"/>
-    <mergeCell ref="AB55:AC55"/>
-    <mergeCell ref="AD55:AE55"/>
-    <mergeCell ref="AF55:AG55"/>
-    <mergeCell ref="AH55:AI55"/>
-    <mergeCell ref="Z54:AA54"/>
-    <mergeCell ref="AB54:AC54"/>
-    <mergeCell ref="AD54:AE54"/>
-    <mergeCell ref="AF54:AG54"/>
-    <mergeCell ref="AH54:AI54"/>
-    <mergeCell ref="Z52:AA52"/>
-    <mergeCell ref="AB52:AC52"/>
-    <mergeCell ref="AD52:AE52"/>
-    <mergeCell ref="AF52:AG52"/>
-    <mergeCell ref="AH52:AI52"/>
-    <mergeCell ref="Z53:AA53"/>
-    <mergeCell ref="AB53:AC53"/>
-    <mergeCell ref="AD53:AE53"/>
-    <mergeCell ref="AF53:AG53"/>
-    <mergeCell ref="AH53:AI53"/>
-    <mergeCell ref="Z50:AA50"/>
-    <mergeCell ref="AB50:AC50"/>
-    <mergeCell ref="AD50:AE50"/>
-    <mergeCell ref="AF50:AG50"/>
-    <mergeCell ref="AH50:AI50"/>
-    <mergeCell ref="Z51:AA51"/>
-    <mergeCell ref="AB51:AC51"/>
-    <mergeCell ref="AD51:AE51"/>
-    <mergeCell ref="AF51:AG51"/>
-    <mergeCell ref="AH51:AI51"/>
-    <mergeCell ref="Z48:AA48"/>
-    <mergeCell ref="AB48:AC48"/>
-    <mergeCell ref="AD48:AE48"/>
-    <mergeCell ref="AF48:AG48"/>
-    <mergeCell ref="AH48:AI48"/>
-    <mergeCell ref="Z49:AA49"/>
-    <mergeCell ref="AB49:AC49"/>
-    <mergeCell ref="AD49:AE49"/>
-    <mergeCell ref="AF49:AG49"/>
-    <mergeCell ref="AH49:AI49"/>
-    <mergeCell ref="Z46:AA46"/>
-    <mergeCell ref="AB46:AC46"/>
-    <mergeCell ref="AD46:AE46"/>
-    <mergeCell ref="AF46:AG46"/>
-    <mergeCell ref="AH46:AI46"/>
-    <mergeCell ref="Z47:AA47"/>
-    <mergeCell ref="AB47:AC47"/>
-    <mergeCell ref="AD47:AE47"/>
-    <mergeCell ref="AF47:AG47"/>
-    <mergeCell ref="AH47:AI47"/>
-    <mergeCell ref="Z44:AA44"/>
-    <mergeCell ref="AB44:AC44"/>
-    <mergeCell ref="AD44:AE44"/>
-    <mergeCell ref="AF44:AG44"/>
-    <mergeCell ref="AH44:AI44"/>
-    <mergeCell ref="Z45:AA45"/>
-    <mergeCell ref="AB45:AC45"/>
-    <mergeCell ref="AD45:AE45"/>
-    <mergeCell ref="AF45:AG45"/>
-    <mergeCell ref="AH45:AI45"/>
-    <mergeCell ref="Z42:AA42"/>
-    <mergeCell ref="AB42:AC42"/>
-    <mergeCell ref="AD42:AE42"/>
-    <mergeCell ref="AF42:AG42"/>
-    <mergeCell ref="AH42:AI42"/>
-    <mergeCell ref="Z43:AA43"/>
-    <mergeCell ref="AB43:AC43"/>
-    <mergeCell ref="AD43:AE43"/>
-    <mergeCell ref="AF43:AG43"/>
-    <mergeCell ref="AH43:AI43"/>
-    <mergeCell ref="Z41:AA41"/>
-    <mergeCell ref="AB41:AC41"/>
-    <mergeCell ref="AD41:AE41"/>
-    <mergeCell ref="AF41:AG41"/>
-    <mergeCell ref="AH41:AI41"/>
+  <mergeCells count="460">
     <mergeCell ref="O54:P54"/>
     <mergeCell ref="Q54:R54"/>
     <mergeCell ref="S54:T54"/>
@@ -14276,7 +14024,7 @@
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="46" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="74" orientation="landscape" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;22ARBEIDSPLAN SIMULATOROPERATØRER</oddHeader>
     <oddFooter>&amp;CUtarbeidet av Stein Mathisen
@@ -17072,10 +16820,10 @@
       </c>
       <c r="O7" s="29"/>
       <c r="P7" s="30"/>
-      <c r="Q7" s="91" t="s">
+      <c r="Q7" s="89" t="s">
         <v>198</v>
       </c>
-      <c r="R7" s="92"/>
+      <c r="R7" s="90"/>
       <c r="S7" s="83"/>
       <c r="T7" s="84"/>
       <c r="U7" s="83"/>
@@ -17112,10 +16860,10 @@
       </c>
       <c r="O8" s="67"/>
       <c r="P8" s="68"/>
-      <c r="Q8" s="91" t="s">
+      <c r="Q8" s="89" t="s">
         <v>198</v>
       </c>
-      <c r="R8" s="92"/>
+      <c r="R8" s="90"/>
       <c r="S8" s="67"/>
       <c r="T8" s="68"/>
       <c r="U8" s="29"/>

</xml_diff>